<commit_message>
feat(billing): GĐ4 phần A – HSTT template convention and template check
- Cell Z1 declares the sheet role (sheet:dntt|dccn|gia-tri|khoi-luong,
  sheet:huong-dan is dropped); buildHstt finds sheets by role, a template
  may hold only some of the 4 sheets, unmarked sheets are copied untouched.
- validateTemplate: unknown placeholders, number placeholders inside text,
  missing/duplicate/non-consecutive row markers, duplicate roles, external
  formulas/links, macros, size > 2MB, charts/shapes/header-footer pictures
  (errors); warnings for the rest.
- Engine: rich-text placeholders, renamed sheets, pictures below the table
  move with the rows, column Z hidden in the output.
- buildEditableTemplate: standard template with markers visible + HUONG_DAN.
- Standard template: Z1 roles added (XML only). T09/2026 Việt Panel fixture
  (800.796.900) + TEST template cases; docs/hstt/cach-tu-lam-mau.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/hstt/hstt-template.xlsx
+++ b/docs/hstt/hstt-template.xlsx
@@ -886,7 +886,13 @@
     <col hidden="1" width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1"/>
+    <row r="1">
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>sheet:dntt</t>
+        </is>
+      </c>
+    </row>
     <row r="2"/>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -1138,7 +1144,13 @@
     <col hidden="1" width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1"/>
+    <row r="1">
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>sheet:dccn</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" s="19" t="inlineStr">
         <is>
@@ -1594,6 +1606,11 @@
           <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM</t>
         </is>
       </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>sheet:gia-tri</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
@@ -2370,7 +2387,13 @@
     <col hidden="1" width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1"/>
+    <row r="1">
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>sheet:khoi-luong</t>
+        </is>
+      </c>
+    </row>
     <row r="2"/>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="19" t="inlineStr">

</xml_diff>